<commit_message>
Fix Mag 7 Feb data: use 2 Feb prices, add --date for backfills
Regenerated MagSeven.xlsx with first trading day (2 Feb) closing
prices instead of 25 Feb. Added --date flag for historical backfills;
normal cron runs use live data which is correct since it only fires
on the 1st-3rd of each month.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/all-in/exports/MagSeven.xlsx
+++ b/projects/all-in/exports/MagSeven.xlsx
@@ -434,13 +434,13 @@
         <v>NVDA</v>
       </c>
       <c r="B3" s="1">
-        <v>196.51</v>
+        <v>185.61</v>
       </c>
       <c r="C3" s="2">
-        <v>4784.4</v>
+        <v>4519</v>
       </c>
       <c r="D3" s="3">
-        <v>0.0793757671370958</v>
+        <v>0.07237522605243935</v>
       </c>
     </row>
     <row r="4">
@@ -448,13 +448,13 @@
         <v>MSFT</v>
       </c>
       <c r="B4" s="1">
-        <v>397.215</v>
+        <v>423.37</v>
       </c>
       <c r="C4" s="2">
-        <v>2949.6</v>
+        <v>3143.8</v>
       </c>
       <c r="D4" s="3">
-        <v>0.048934681930963606</v>
+        <v>0.050349653501720465</v>
       </c>
     </row>
     <row r="5">
@@ -462,13 +462,13 @@
         <v>AAPL</v>
       </c>
       <c r="B5" s="1">
-        <v>274.265</v>
+        <v>270.01</v>
       </c>
       <c r="C5" s="2">
-        <v>4031.1</v>
+        <v>3968.6</v>
       </c>
       <c r="D5" s="3">
-        <v>0.06687814832728885</v>
+        <v>0.06355928405907679</v>
       </c>
     </row>
     <row r="6">
@@ -476,13 +476,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B6" s="1">
-        <v>309.58</v>
+        <v>343.69</v>
       </c>
       <c r="C6" s="2">
-        <v>3745</v>
+        <v>4157.6</v>
       </c>
       <c r="D6" s="3">
-        <v>0.062131013190170795</v>
+        <v>0.06658673497962327</v>
       </c>
     </row>
     <row r="7">
@@ -490,13 +490,13 @@
         <v>AMZN</v>
       </c>
       <c r="B7" s="1">
-        <v>209.88</v>
+        <v>242.96</v>
       </c>
       <c r="C7" s="2">
-        <v>2253</v>
+        <v>2608.2</v>
       </c>
       <c r="D7" s="3">
-        <v>0.03737893148560992</v>
+        <v>0.04177109872942263</v>
       </c>
     </row>
     <row r="8">
@@ -504,13 +504,13 @@
         <v>META</v>
       </c>
       <c r="B8" s="1">
-        <v>648.035</v>
+        <v>706.41</v>
       </c>
       <c r="C8" s="2">
-        <v>1633.7</v>
+        <v>1780.9</v>
       </c>
       <c r="D8" s="3">
-        <v>0.027103658753192747</v>
+        <v>0.028521447405085734</v>
       </c>
     </row>
     <row r="9">
@@ -518,13 +518,13 @@
         <v>TSLA</v>
       </c>
       <c r="B9" s="1">
-        <v>414.86</v>
+        <v>421.81</v>
       </c>
       <c r="C9" s="2">
-        <v>1556.7</v>
+        <v>1582.8</v>
       </c>
       <c r="D9" s="3">
-        <v>0.02582689612571888</v>
+        <v>0.025349698762714624</v>
       </c>
     </row>
     <row r="10">
@@ -532,10 +532,10 @@
         <v>TOTAL</v>
       </c>
       <c r="C10" s="2">
-        <v>20953.6</v>
+        <v>21760.9</v>
       </c>
       <c r="D10" s="3">
-        <v>0.34762909695004063</v>
+        <v>0.34851314349008283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backfill January 2026 Mag 7 data (2 Jan prices)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/all-in/exports/MagSeven.xlsx
+++ b/projects/all-in/exports/MagSeven.xlsx
@@ -402,13 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -433,13 +427,13 @@
       <c r="A3" t="str">
         <v>NVDA</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3">
         <v>185.61</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3">
         <v>4519</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
         <v>0.07237522605243935</v>
       </c>
     </row>
@@ -447,13 +441,13 @@
       <c r="A4" t="str">
         <v>MSFT</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4">
         <v>423.37</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4">
         <v>3143.8</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
         <v>0.050349653501720465</v>
       </c>
     </row>
@@ -461,13 +455,13 @@
       <c r="A5" t="str">
         <v>AAPL</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>270.01</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>3968.6</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
         <v>0.06355928405907679</v>
       </c>
     </row>
@@ -475,13 +469,13 @@
       <c r="A6" t="str">
         <v>GOOGL</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6">
         <v>343.69</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>4157.6</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6">
         <v>0.06658673497962327</v>
       </c>
     </row>
@@ -489,13 +483,13 @@
       <c r="A7" t="str">
         <v>AMZN</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7">
         <v>242.96</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7">
         <v>2608.2</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7">
         <v>0.04177109872942263</v>
       </c>
     </row>
@@ -503,13 +497,13 @@
       <c r="A8" t="str">
         <v>META</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8">
         <v>706.41</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8">
         <v>1780.9</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8">
         <v>0.028521447405085734</v>
       </c>
     </row>
@@ -517,13 +511,13 @@
       <c r="A9" t="str">
         <v>TSLA</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9">
         <v>421.81</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9">
         <v>1582.8</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9">
         <v>0.025349698762714624</v>
       </c>
     </row>
@@ -531,19 +525,148 @@
       <c r="A10" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10">
         <v>21760.9</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10">
         <v>0.34851314349008283</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>January 2026</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B14" s="1">
+        <v>188.85</v>
+      </c>
+      <c r="C14" s="2">
+        <v>4597.9</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.07490523435884068</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B15" s="1">
+        <v>472.94</v>
+      </c>
+      <c r="C15" s="2">
+        <v>3511.9</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.057212254610596876</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B16" s="1">
+        <v>271.01</v>
+      </c>
+      <c r="C16" s="2">
+        <v>3983.3</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.06489198615336658</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B17" s="1">
+        <v>315.15</v>
+      </c>
+      <c r="C17" s="2">
+        <v>3812.4</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.062107597094422165</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B18" s="1">
+        <v>226.5</v>
+      </c>
+      <c r="C18" s="2">
+        <v>2431.5</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.03961101010148268</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>META</v>
+      </c>
+      <c r="B19" s="1">
+        <v>650.41</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1639.7</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.026712130893460088</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B20" s="1">
+        <v>438.07</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1643.8</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.02677972153913024</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C21" s="2">
+        <v>21620.4</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.35221993475129937</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Backfill Mag 7 data for all of 2025
12 months of first-trading-day snapshots. Mag 7 ranged from 30.4%
(April, tariff selloff) to 36.5% (November) of S&P 500.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/all-in/exports/MagSeven.xlsx
+++ b/projects/all-in/exports/MagSeven.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D153"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -555,13 +555,13 @@
       <c r="A14" t="str">
         <v>NVDA</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14">
         <v>188.85</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14">
         <v>4597.9</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14">
         <v>0.07490523435884068</v>
       </c>
     </row>
@@ -569,13 +569,13 @@
       <c r="A15" t="str">
         <v>MSFT</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15">
         <v>472.94</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15">
         <v>3511.9</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15">
         <v>0.057212254610596876</v>
       </c>
     </row>
@@ -583,13 +583,13 @@
       <c r="A16" t="str">
         <v>AAPL</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16">
         <v>271.01</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16">
         <v>3983.3</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16">
         <v>0.06489198615336658</v>
       </c>
     </row>
@@ -597,13 +597,13 @@
       <c r="A17" t="str">
         <v>GOOGL</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17">
         <v>315.15</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17">
         <v>3812.4</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17">
         <v>0.062107597094422165</v>
       </c>
     </row>
@@ -611,13 +611,13 @@
       <c r="A18" t="str">
         <v>AMZN</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18">
         <v>226.5</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18">
         <v>2431.5</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18">
         <v>0.03961101010148268</v>
       </c>
     </row>
@@ -625,13 +625,13 @@
       <c r="A19" t="str">
         <v>META</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19">
         <v>650.41</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19">
         <v>1639.7</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19">
         <v>0.026712130893460088</v>
       </c>
     </row>
@@ -639,13 +639,13 @@
       <c r="A20" t="str">
         <v>TSLA</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20">
         <v>438.07</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>1643.8</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20">
         <v>0.02677972153913024</v>
       </c>
     </row>
@@ -653,20 +653,1568 @@
       <c r="A21" t="str">
         <v>TOTAL</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21">
         <v>21620.4</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21">
         <v>0.35221993475129937</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>January 2025</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D24" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B25">
+        <v>138.31</v>
+      </c>
+      <c r="C25">
+        <v>3367.4</v>
+      </c>
+      <c r="D25">
+        <v>0.06411286725772856</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B26">
+        <v>418.58</v>
+      </c>
+      <c r="C26">
+        <v>3108.2</v>
+      </c>
+      <c r="D26">
+        <v>0.059177680041089614</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B27">
+        <v>243.85</v>
+      </c>
+      <c r="C27">
+        <v>3584.1</v>
+      </c>
+      <c r="D27">
+        <v>0.06823779236125156</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B28">
+        <v>189.43</v>
+      </c>
+      <c r="C28">
+        <v>2291.5</v>
+      </c>
+      <c r="D28">
+        <v>0.04362873577281996</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B29">
+        <v>220.22</v>
+      </c>
+      <c r="C29">
+        <v>2364</v>
+      </c>
+      <c r="D29">
+        <v>0.04500916270005028</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>META</v>
+      </c>
+      <c r="B30">
+        <v>599.24</v>
+      </c>
+      <c r="C30">
+        <v>1510.7</v>
+      </c>
+      <c r="D30">
+        <v>0.02876196760035955</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B31">
+        <v>379.28</v>
+      </c>
+      <c r="C31">
+        <v>1423.2</v>
+      </c>
+      <c r="D31">
+        <v>0.02709685828244846</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C32">
+        <v>17649.2</v>
+      </c>
+      <c r="D32">
+        <v>0.336025064015748</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>February 2025</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B36">
+        <v>116.66</v>
+      </c>
+      <c r="C36">
+        <v>2840.3</v>
+      </c>
+      <c r="D36">
+        <v>0.05294029821847482</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B37">
+        <v>410.92</v>
+      </c>
+      <c r="C37">
+        <v>3051.3</v>
+      </c>
+      <c r="D37">
+        <v>0.05687344567848971</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B38">
+        <v>228.01</v>
+      </c>
+      <c r="C38">
+        <v>3351.3</v>
+      </c>
+      <c r="D38">
+        <v>0.06246386497163106</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B39">
+        <v>201.23</v>
+      </c>
+      <c r="C39">
+        <v>2434.3</v>
+      </c>
+      <c r="D39">
+        <v>0.04537215171748848</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B40">
+        <v>237.42</v>
+      </c>
+      <c r="C40">
+        <v>2548.7</v>
+      </c>
+      <c r="D40">
+        <v>0.04750444427961135</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>META</v>
+      </c>
+      <c r="B41">
+        <v>697.46</v>
+      </c>
+      <c r="C41">
+        <v>1758.3</v>
+      </c>
+      <c r="D41">
+        <v>0.03277252436939172</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B42">
+        <v>383.68</v>
+      </c>
+      <c r="C42">
+        <v>1439.7</v>
+      </c>
+      <c r="D42">
+        <v>0.02683495823227238</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C43">
+        <v>17423.9</v>
+      </c>
+      <c r="D43">
+        <v>0.3247616874673595</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>March 2025</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D46" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B47">
+        <v>114.06</v>
+      </c>
+      <c r="C47">
+        <v>2777</v>
+      </c>
+      <c r="D47">
+        <v>0.053042096830427356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B48">
+        <v>388.49</v>
+      </c>
+      <c r="C48">
+        <v>2884.8</v>
+      </c>
+      <c r="D48">
+        <v>0.05510043263941791</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B49">
+        <v>238.03</v>
+      </c>
+      <c r="C49">
+        <v>3498.5</v>
+      </c>
+      <c r="D49">
+        <v>0.06682355733740863</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B50">
+        <v>167.01</v>
+      </c>
+      <c r="C50">
+        <v>2020.3</v>
+      </c>
+      <c r="D50">
+        <v>0.03858886880058495</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B51">
+        <v>205.02</v>
+      </c>
+      <c r="C51">
+        <v>2200.9</v>
+      </c>
+      <c r="D51">
+        <v>0.042037425561212205</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>META</v>
+      </c>
+      <c r="B52">
+        <v>655.05</v>
+      </c>
+      <c r="C52">
+        <v>1651.4</v>
+      </c>
+      <c r="D52">
+        <v>0.0315419070226463</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B53">
+        <v>284.65</v>
+      </c>
+      <c r="C53">
+        <v>1068.1</v>
+      </c>
+      <c r="D53">
+        <v>0.02040167748110477</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C54">
+        <v>16101</v>
+      </c>
+      <c r="D54">
+        <v>0.3075359656728021</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>April 2025</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D57" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B58">
+        <v>110.15</v>
+      </c>
+      <c r="C58">
+        <v>2681.8</v>
+      </c>
+      <c r="D58">
+        <v>0.05339503390497378</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B59">
+        <v>382.19</v>
+      </c>
+      <c r="C59">
+        <v>2838</v>
+      </c>
+      <c r="D59">
+        <v>0.05650456435770747</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B60">
+        <v>223.19</v>
+      </c>
+      <c r="C60">
+        <v>3280.4</v>
+      </c>
+      <c r="D60">
+        <v>0.06531330597781751</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B61">
+        <v>157.07</v>
+      </c>
+      <c r="C61">
+        <v>1900.1</v>
+      </c>
+      <c r="D61">
+        <v>0.03783048273057432</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B62">
+        <v>192.17</v>
+      </c>
+      <c r="C62">
+        <v>2062.9</v>
+      </c>
+      <c r="D62">
+        <v>0.041072817181503976</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>META</v>
+      </c>
+      <c r="B63">
+        <v>586</v>
+      </c>
+      <c r="C63">
+        <v>1477.3</v>
+      </c>
+      <c r="D63">
+        <v>0.02941305624329163</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B64">
+        <v>268.46</v>
+      </c>
+      <c r="C64">
+        <v>1007.4</v>
+      </c>
+      <c r="D64">
+        <v>0.020056876668653946</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C65">
+        <v>15247.9</v>
+      </c>
+      <c r="D65">
+        <v>0.30358613706452264</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>May 2025</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D68" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B69">
+        <v>111.61</v>
+      </c>
+      <c r="C69">
+        <v>2717.4</v>
+      </c>
+      <c r="D69">
+        <v>0.05451846630102624</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B70">
+        <v>425.4</v>
+      </c>
+      <c r="C70">
+        <v>3158.9</v>
+      </c>
+      <c r="D70">
+        <v>0.06337614930315627</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B71">
+        <v>213.32</v>
+      </c>
+      <c r="C71">
+        <v>3135.4</v>
+      </c>
+      <c r="D71">
+        <v>0.06290463986676066</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B72">
+        <v>161.3</v>
+      </c>
+      <c r="C72">
+        <v>1951.2</v>
+      </c>
+      <c r="D72">
+        <v>0.039147781434829075</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B73">
+        <v>190.2</v>
+      </c>
+      <c r="C73">
+        <v>2041.8</v>
+      </c>
+      <c r="D73">
+        <v>0.040964114557301146</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>META</v>
+      </c>
+      <c r="B74">
+        <v>572.21</v>
+      </c>
+      <c r="C74">
+        <v>1442.5</v>
+      </c>
+      <c r="D74">
+        <v>0.028941574726441665</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B75">
+        <v>280.52</v>
+      </c>
+      <c r="C75">
+        <v>1052.6</v>
+      </c>
+      <c r="D75">
+        <v>0.021118920018962154</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C76">
+        <v>15499.8</v>
+      </c>
+      <c r="D76">
+        <v>0.3109716462084772</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>June 2025</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D79" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B80">
+        <v>137.38</v>
+      </c>
+      <c r="C80">
+        <v>3344.8</v>
+      </c>
+      <c r="D80">
+        <v>0.06295880121805197</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B81">
+        <v>461.97</v>
+      </c>
+      <c r="C81">
+        <v>3430.4</v>
+      </c>
+      <c r="D81">
+        <v>0.06457055911880254</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B82">
+        <v>201.7</v>
+      </c>
+      <c r="C82">
+        <v>2964.6</v>
+      </c>
+      <c r="D82">
+        <v>0.05580195124854954</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B83">
+        <v>169.03</v>
+      </c>
+      <c r="C83">
+        <v>2044.8</v>
+      </c>
+      <c r="D83">
+        <v>0.03848832144017101</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B84">
+        <v>206.65</v>
+      </c>
+      <c r="C84">
+        <v>2218.4</v>
+      </c>
+      <c r="D84">
+        <v>0.04175619013332163</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>META</v>
+      </c>
+      <c r="B85">
+        <v>670.9</v>
+      </c>
+      <c r="C85">
+        <v>1691.3</v>
+      </c>
+      <c r="D85">
+        <v>0.03183588363426788</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B86">
+        <v>342.69</v>
+      </c>
+      <c r="C86">
+        <v>1285.9</v>
+      </c>
+      <c r="D86">
+        <v>0.02420481291007333</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C87">
+        <v>16980.2</v>
+      </c>
+      <c r="D87">
+        <v>0.3196165197032379</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>July 2025</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D90" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B91">
+        <v>153.3</v>
+      </c>
+      <c r="C91">
+        <v>3732.4</v>
+      </c>
+      <c r="D91">
+        <v>0.06720882215989255</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B92">
+        <v>492.05</v>
+      </c>
+      <c r="C92">
+        <v>3653.8</v>
+      </c>
+      <c r="D92">
+        <v>0.06579322817362217</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B93">
+        <v>207.82</v>
+      </c>
+      <c r="C93">
+        <v>3054.5</v>
+      </c>
+      <c r="D93">
+        <v>0.055002451626620034</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B94">
+        <v>175.84</v>
+      </c>
+      <c r="C94">
+        <v>2127.1</v>
+      </c>
+      <c r="D94">
+        <v>0.03830311081425009</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B95">
+        <v>220.46</v>
+      </c>
+      <c r="C95">
+        <v>2366.6</v>
+      </c>
+      <c r="D95">
+        <v>0.04261539165957815</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>META</v>
+      </c>
+      <c r="B96">
+        <v>719.22</v>
+      </c>
+      <c r="C96">
+        <v>1813.1</v>
+      </c>
+      <c r="D96">
+        <v>0.032649161880347714</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B97">
+        <v>300.71</v>
+      </c>
+      <c r="C97">
+        <v>1128.4</v>
+      </c>
+      <c r="D97">
+        <v>0.020318860659609094</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C98">
+        <v>17876</v>
+      </c>
+      <c r="D98">
+        <v>0.3218910269739198</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>August 2025</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D101" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B102">
+        <v>173.72</v>
+      </c>
+      <c r="C102">
+        <v>4229.6</v>
+      </c>
+      <c r="D102">
+        <v>0.07454607206092621</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B103">
+        <v>524.11</v>
+      </c>
+      <c r="C103">
+        <v>3891.8</v>
+      </c>
+      <c r="D103">
+        <v>0.06859385712344067</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B104">
+        <v>202.38</v>
+      </c>
+      <c r="C104">
+        <v>2974.6</v>
+      </c>
+      <c r="D104">
+        <v>0.052426771494219315</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B105">
+        <v>189.13</v>
+      </c>
+      <c r="C105">
+        <v>2287.9</v>
+      </c>
+      <c r="D105">
+        <v>0.040324374067196835</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B106">
+        <v>214.75</v>
+      </c>
+      <c r="C106">
+        <v>2305.3</v>
+      </c>
+      <c r="D106">
+        <v>0.040631294641370906</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>META</v>
+      </c>
+      <c r="B107">
+        <v>750.01</v>
+      </c>
+      <c r="C107">
+        <v>1890.8</v>
+      </c>
+      <c r="D107">
+        <v>0.033324848131571445</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B108">
+        <v>302.63</v>
+      </c>
+      <c r="C108">
+        <v>1135.6</v>
+      </c>
+      <c r="D108">
+        <v>0.020014940287187883</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C109">
+        <v>18715.6</v>
+      </c>
+      <c r="D109">
+        <v>0.3298621578059132</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>September 2025</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C112" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D112" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B113">
+        <v>170.78</v>
+      </c>
+      <c r="C113">
+        <v>4158</v>
+      </c>
+      <c r="D113">
+        <v>0.07241461186451607</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B114">
+        <v>505.12</v>
+      </c>
+      <c r="C114">
+        <v>3750.8</v>
+      </c>
+      <c r="D114">
+        <v>0.06532382564354466</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B115">
+        <v>229.72</v>
+      </c>
+      <c r="C115">
+        <v>3376.4</v>
+      </c>
+      <c r="D115">
+        <v>0.058802877963955745</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B116">
+        <v>211.35</v>
+      </c>
+      <c r="C116">
+        <v>2556.7</v>
+      </c>
+      <c r="D116">
+        <v>0.04452702975580989</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B117">
+        <v>225.34</v>
+      </c>
+      <c r="C117">
+        <v>2419</v>
+      </c>
+      <c r="D117">
+        <v>0.042128891399379656</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>META</v>
+      </c>
+      <c r="B118">
+        <v>735.11</v>
+      </c>
+      <c r="C118">
+        <v>1853.2</v>
+      </c>
+      <c r="D118">
+        <v>0.03227510779350659</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B119">
+        <v>329.36</v>
+      </c>
+      <c r="C119">
+        <v>1235.9</v>
+      </c>
+      <c r="D119">
+        <v>0.021524219321961406</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C120">
+        <v>19350</v>
+      </c>
+      <c r="D120">
+        <v>0.336996563742674</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>October 2025</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C123" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D123" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B124">
+        <v>187.24</v>
+      </c>
+      <c r="C124">
+        <v>4558.7</v>
+      </c>
+      <c r="D124">
+        <v>0.07615438836911599</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B125">
+        <v>519.71</v>
+      </c>
+      <c r="C125">
+        <v>3859.2</v>
+      </c>
+      <c r="D125">
+        <v>0.0644681533775499</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B126">
+        <v>255.45</v>
+      </c>
+      <c r="C126">
+        <v>3754.6</v>
+      </c>
+      <c r="D126">
+        <v>0.06272096940724874</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B127">
+        <v>244.9</v>
+      </c>
+      <c r="C127">
+        <v>2962.6</v>
+      </c>
+      <c r="D127">
+        <v>0.049489985154853276</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B128">
+        <v>220.63</v>
+      </c>
+      <c r="C128">
+        <v>2368.4</v>
+      </c>
+      <c r="D128">
+        <v>0.039565204139548324</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>META</v>
+      </c>
+      <c r="B129">
+        <v>717.34</v>
+      </c>
+      <c r="C129">
+        <v>1808.4</v>
+      </c>
+      <c r="D129">
+        <v>0.03020977788937343</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B130">
+        <v>459.46</v>
+      </c>
+      <c r="C130">
+        <v>1724.1</v>
+      </c>
+      <c r="D130">
+        <v>0.028801251680996544</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C131">
+        <v>21036</v>
+      </c>
+      <c r="D131">
+        <v>0.35140973001868625</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>November 2025</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C134" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D134" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B135">
+        <v>206.88</v>
+      </c>
+      <c r="C135">
+        <v>5036.9</v>
+      </c>
+      <c r="D135">
+        <v>0.08213447248644803</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B136">
+        <v>517.03</v>
+      </c>
+      <c r="C136">
+        <v>3839.3</v>
+      </c>
+      <c r="D136">
+        <v>0.0626052237012684</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B137">
+        <v>269.05</v>
+      </c>
+      <c r="C137">
+        <v>3954.5</v>
+      </c>
+      <c r="D137">
+        <v>0.0644837821548035</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B138">
+        <v>283.72</v>
+      </c>
+      <c r="C138">
+        <v>3432.2</v>
+      </c>
+      <c r="D138">
+        <v>0.05596663135977788</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B139">
+        <v>254</v>
+      </c>
+      <c r="C139">
+        <v>2726.7</v>
+      </c>
+      <c r="D139">
+        <v>0.04446243241248235</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>META</v>
+      </c>
+      <c r="B140">
+        <v>637.71</v>
+      </c>
+      <c r="C140">
+        <v>1607.7</v>
+      </c>
+      <c r="D140">
+        <v>0.026215393133655042</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B141">
+        <v>468.37</v>
+      </c>
+      <c r="C141">
+        <v>1757.5</v>
+      </c>
+      <c r="D141">
+        <v>0.028659155747857726</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C142">
+        <v>22354.7</v>
+      </c>
+      <c r="D142">
+        <v>0.36452709099629294</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>December 2025</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C145" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D145" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B146" s="1">
+        <v>179.92</v>
+      </c>
+      <c r="C146" s="2">
+        <v>4380.5</v>
+      </c>
+      <c r="D146" s="3">
+        <v>0.07184343084835443</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B147" s="1">
+        <v>486.74</v>
+      </c>
+      <c r="C147" s="2">
+        <v>3614.4</v>
+      </c>
+      <c r="D147" s="3">
+        <v>0.05927785829233961</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B148" s="1">
+        <v>283.1</v>
+      </c>
+      <c r="C148" s="2">
+        <v>4161</v>
+      </c>
+      <c r="D148" s="3">
+        <v>0.06824299450538433</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B149" s="1">
+        <v>314.89</v>
+      </c>
+      <c r="C149" s="2">
+        <v>3809.2</v>
+      </c>
+      <c r="D149" s="3">
+        <v>0.06247392253795553</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B150" s="1">
+        <v>233.88</v>
+      </c>
+      <c r="C150" s="2">
+        <v>2510.7</v>
+      </c>
+      <c r="D150" s="3">
+        <v>0.04117686389540775</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>META</v>
+      </c>
+      <c r="B151" s="1">
+        <v>640.87</v>
+      </c>
+      <c r="C151" s="2">
+        <v>1615.6</v>
+      </c>
+      <c r="D151" s="3">
+        <v>0.026497429343704814</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B152" s="1">
+        <v>430.14</v>
+      </c>
+      <c r="C152" s="2">
+        <v>1614.1</v>
+      </c>
+      <c r="D152" s="3">
+        <v>0.026471883574073173</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C153" s="2">
+        <v>21705.4</v>
+      </c>
+      <c r="D153" s="3">
+        <v>0.35598438299721963</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="14">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="A78:D78"/>
+    <mergeCell ref="A89:D89"/>
+    <mergeCell ref="A100:D100"/>
+    <mergeCell ref="A111:D111"/>
+    <mergeCell ref="A122:D122"/>
+    <mergeCell ref="A133:D133"/>
+    <mergeCell ref="A144:D144"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D153"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild MagSeven.xlsx in chronological order (oldest first)
New months append at the bottom, extending the timeline naturally
for graphing. Includes June 2025 which was missing from prior build.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/all-in/exports/MagSeven.xlsx
+++ b/projects/all-in/exports/MagSeven.xlsx
@@ -406,7 +406,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>February 2026</v>
+        <v>January 2025</v>
       </c>
     </row>
     <row r="2">
@@ -428,13 +428,13 @@
         <v>NVDA</v>
       </c>
       <c r="B3">
-        <v>185.61</v>
+        <v>138.31</v>
       </c>
       <c r="C3">
-        <v>4519</v>
+        <v>3367.4</v>
       </c>
       <c r="D3">
-        <v>0.07237522605243935</v>
+        <v>0.06411286725772856</v>
       </c>
     </row>
     <row r="4">
@@ -442,13 +442,13 @@
         <v>MSFT</v>
       </c>
       <c r="B4">
-        <v>423.37</v>
+        <v>418.58</v>
       </c>
       <c r="C4">
-        <v>3143.8</v>
+        <v>3108.2</v>
       </c>
       <c r="D4">
-        <v>0.050349653501720465</v>
+        <v>0.059177680041089614</v>
       </c>
     </row>
     <row r="5">
@@ -456,13 +456,13 @@
         <v>AAPL</v>
       </c>
       <c r="B5">
-        <v>270.01</v>
+        <v>243.85</v>
       </c>
       <c r="C5">
-        <v>3968.6</v>
+        <v>3584.1</v>
       </c>
       <c r="D5">
-        <v>0.06355928405907679</v>
+        <v>0.06823779236125156</v>
       </c>
     </row>
     <row r="6">
@@ -470,13 +470,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B6">
-        <v>343.69</v>
+        <v>189.43</v>
       </c>
       <c r="C6">
-        <v>4157.6</v>
+        <v>2291.5</v>
       </c>
       <c r="D6">
-        <v>0.06658673497962327</v>
+        <v>0.04362873491806178</v>
       </c>
     </row>
     <row r="7">
@@ -484,13 +484,13 @@
         <v>AMZN</v>
       </c>
       <c r="B7">
-        <v>242.96</v>
+        <v>220.22</v>
       </c>
       <c r="C7">
-        <v>2608.2</v>
+        <v>2364</v>
       </c>
       <c r="D7">
-        <v>0.04177109872942263</v>
+        <v>0.04500916270005028</v>
       </c>
     </row>
     <row r="8">
@@ -498,13 +498,13 @@
         <v>META</v>
       </c>
       <c r="B8">
-        <v>706.41</v>
+        <v>599.24</v>
       </c>
       <c r="C8">
-        <v>1780.9</v>
+        <v>1510.7</v>
       </c>
       <c r="D8">
-        <v>0.028521447405085734</v>
+        <v>0.02876196760035955</v>
       </c>
     </row>
     <row r="9">
@@ -512,13 +512,13 @@
         <v>TSLA</v>
       </c>
       <c r="B9">
-        <v>421.81</v>
+        <v>379.28</v>
       </c>
       <c r="C9">
-        <v>1582.8</v>
+        <v>1423.2</v>
       </c>
       <c r="D9">
-        <v>0.025349698762714624</v>
+        <v>0.02709685828244846</v>
       </c>
     </row>
     <row r="10">
@@ -526,15 +526,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C10">
-        <v>21760.9</v>
+        <v>17649.2</v>
       </c>
       <c r="D10">
-        <v>0.34851314349008283</v>
+        <v>0.3360250631609898</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>January 2026</v>
+        <v>February 2025</v>
       </c>
     </row>
     <row r="13">
@@ -556,13 +556,13 @@
         <v>NVDA</v>
       </c>
       <c r="B14">
-        <v>188.85</v>
+        <v>116.66</v>
       </c>
       <c r="C14">
-        <v>4597.9</v>
+        <v>2840.3</v>
       </c>
       <c r="D14">
-        <v>0.07490523435884068</v>
+        <v>0.05294029821847482</v>
       </c>
     </row>
     <row r="15">
@@ -570,13 +570,13 @@
         <v>MSFT</v>
       </c>
       <c r="B15">
-        <v>472.94</v>
+        <v>410.92</v>
       </c>
       <c r="C15">
-        <v>3511.9</v>
+        <v>3051.3</v>
       </c>
       <c r="D15">
-        <v>0.057212254610596876</v>
+        <v>0.05687344567848971</v>
       </c>
     </row>
     <row r="16">
@@ -584,13 +584,13 @@
         <v>AAPL</v>
       </c>
       <c r="B16">
-        <v>271.01</v>
+        <v>228.01</v>
       </c>
       <c r="C16">
-        <v>3983.3</v>
+        <v>3351.3</v>
       </c>
       <c r="D16">
-        <v>0.06489198615336658</v>
+        <v>0.06246386497163106</v>
       </c>
     </row>
     <row r="17">
@@ -598,13 +598,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B17">
-        <v>315.15</v>
+        <v>201.23</v>
       </c>
       <c r="C17">
-        <v>3812.4</v>
+        <v>2434.3</v>
       </c>
       <c r="D17">
-        <v>0.062107597094422165</v>
+        <v>0.04537215082857395</v>
       </c>
     </row>
     <row r="18">
@@ -612,13 +612,13 @@
         <v>AMZN</v>
       </c>
       <c r="B18">
-        <v>226.5</v>
+        <v>237.42</v>
       </c>
       <c r="C18">
-        <v>2431.5</v>
+        <v>2548.7</v>
       </c>
       <c r="D18">
-        <v>0.03961101010148268</v>
+        <v>0.04750444427961135</v>
       </c>
     </row>
     <row r="19">
@@ -626,13 +626,13 @@
         <v>META</v>
       </c>
       <c r="B19">
-        <v>650.41</v>
+        <v>697.46</v>
       </c>
       <c r="C19">
-        <v>1639.7</v>
+        <v>1758.3</v>
       </c>
       <c r="D19">
-        <v>0.026712130893460088</v>
+        <v>0.03277252436939172</v>
       </c>
     </row>
     <row r="20">
@@ -640,13 +640,13 @@
         <v>TSLA</v>
       </c>
       <c r="B20">
-        <v>438.07</v>
+        <v>383.68</v>
       </c>
       <c r="C20">
-        <v>1643.8</v>
+        <v>1439.7</v>
       </c>
       <c r="D20">
-        <v>0.02677972153913024</v>
+        <v>0.02683495823227238</v>
       </c>
     </row>
     <row r="21">
@@ -654,15 +654,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C21">
-        <v>21620.4</v>
+        <v>17423.9</v>
       </c>
       <c r="D21">
-        <v>0.35221993475129937</v>
+        <v>0.32476168657844495</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>January 2025</v>
+        <v>March 2025</v>
       </c>
     </row>
     <row r="24">
@@ -684,13 +684,13 @@
         <v>NVDA</v>
       </c>
       <c r="B25">
-        <v>138.31</v>
+        <v>114.06</v>
       </c>
       <c r="C25">
-        <v>3367.4</v>
+        <v>2777</v>
       </c>
       <c r="D25">
-        <v>0.06411286725772856</v>
+        <v>0.053042096830427356</v>
       </c>
     </row>
     <row r="26">
@@ -698,13 +698,13 @@
         <v>MSFT</v>
       </c>
       <c r="B26">
-        <v>418.58</v>
+        <v>388.49</v>
       </c>
       <c r="C26">
-        <v>3108.2</v>
+        <v>2884.8</v>
       </c>
       <c r="D26">
-        <v>0.059177680041089614</v>
+        <v>0.05510043263941791</v>
       </c>
     </row>
     <row r="27">
@@ -712,13 +712,13 @@
         <v>AAPL</v>
       </c>
       <c r="B27">
-        <v>243.85</v>
+        <v>238.03</v>
       </c>
       <c r="C27">
-        <v>3584.1</v>
+        <v>3498.5</v>
       </c>
       <c r="D27">
-        <v>0.06823779236125156</v>
+        <v>0.06682355733740863</v>
       </c>
     </row>
     <row r="28">
@@ -726,13 +726,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B28">
-        <v>189.43</v>
+        <v>167.01</v>
       </c>
       <c r="C28">
-        <v>2291.5</v>
+        <v>2020.3</v>
       </c>
       <c r="D28">
-        <v>0.04362873577281996</v>
+        <v>0.03858886804456601</v>
       </c>
     </row>
     <row r="29">
@@ -740,13 +740,13 @@
         <v>AMZN</v>
       </c>
       <c r="B29">
-        <v>220.22</v>
+        <v>205.02</v>
       </c>
       <c r="C29">
-        <v>2364</v>
+        <v>2200.9</v>
       </c>
       <c r="D29">
-        <v>0.04500916270005028</v>
+        <v>0.042037425561212205</v>
       </c>
     </row>
     <row r="30">
@@ -754,13 +754,13 @@
         <v>META</v>
       </c>
       <c r="B30">
-        <v>599.24</v>
+        <v>655.05</v>
       </c>
       <c r="C30">
-        <v>1510.7</v>
+        <v>1651.4</v>
       </c>
       <c r="D30">
-        <v>0.02876196760035955</v>
+        <v>0.0315419070226463</v>
       </c>
     </row>
     <row r="31">
@@ -768,13 +768,13 @@
         <v>TSLA</v>
       </c>
       <c r="B31">
-        <v>379.28</v>
+        <v>284.65</v>
       </c>
       <c r="C31">
-        <v>1423.2</v>
+        <v>1068.1</v>
       </c>
       <c r="D31">
-        <v>0.02709685828244846</v>
+        <v>0.02040167748110477</v>
       </c>
     </row>
     <row r="32">
@@ -782,15 +782,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C32">
-        <v>17649.2</v>
+        <v>16101</v>
       </c>
       <c r="D32">
-        <v>0.336025064015748</v>
+        <v>0.30753596491678314</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>February 2025</v>
+        <v>April 2025</v>
       </c>
     </row>
     <row r="35">
@@ -812,13 +812,13 @@
         <v>NVDA</v>
       </c>
       <c r="B36">
-        <v>116.66</v>
+        <v>110.15</v>
       </c>
       <c r="C36">
-        <v>2840.3</v>
+        <v>0</v>
       </c>
       <c r="D36">
-        <v>0.05294029821847482</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -826,13 +826,13 @@
         <v>MSFT</v>
       </c>
       <c r="B37">
-        <v>410.92</v>
+        <v>382.19</v>
       </c>
       <c r="C37">
-        <v>3051.3</v>
+        <v>0</v>
       </c>
       <c r="D37">
-        <v>0.05687344567848971</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -840,13 +840,13 @@
         <v>AAPL</v>
       </c>
       <c r="B38">
-        <v>228.01</v>
+        <v>223.19</v>
       </c>
       <c r="C38">
-        <v>3351.3</v>
+        <v>0</v>
       </c>
       <c r="D38">
-        <v>0.06246386497163106</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -854,13 +854,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B39">
-        <v>201.23</v>
+        <v>157.07</v>
       </c>
       <c r="C39">
-        <v>2434.3</v>
+        <v>0</v>
       </c>
       <c r="D39">
-        <v>0.04537215171748848</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -868,13 +868,13 @@
         <v>AMZN</v>
       </c>
       <c r="B40">
-        <v>237.42</v>
+        <v>192.17</v>
       </c>
       <c r="C40">
-        <v>2548.7</v>
+        <v>0</v>
       </c>
       <c r="D40">
-        <v>0.04750444427961135</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -882,13 +882,13 @@
         <v>META</v>
       </c>
       <c r="B41">
-        <v>697.46</v>
+        <v>586</v>
       </c>
       <c r="C41">
-        <v>1758.3</v>
+        <v>0</v>
       </c>
       <c r="D41">
-        <v>0.03277252436939172</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -896,13 +896,13 @@
         <v>TSLA</v>
       </c>
       <c r="B42">
-        <v>383.68</v>
+        <v>268.46</v>
       </c>
       <c r="C42">
-        <v>1439.7</v>
+        <v>0</v>
       </c>
       <c r="D42">
-        <v>0.02683495823227238</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -910,15 +910,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C43">
-        <v>17423.9</v>
+        <v>0</v>
       </c>
       <c r="D43">
-        <v>0.3247616874673595</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>March 2025</v>
+        <v>May 2025</v>
       </c>
     </row>
     <row r="46">
@@ -940,13 +940,13 @@
         <v>NVDA</v>
       </c>
       <c r="B47">
-        <v>114.06</v>
+        <v>111.61</v>
       </c>
       <c r="C47">
-        <v>2777</v>
+        <v>0</v>
       </c>
       <c r="D47">
-        <v>0.053042096830427356</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -954,13 +954,13 @@
         <v>MSFT</v>
       </c>
       <c r="B48">
-        <v>388.49</v>
+        <v>425.4</v>
       </c>
       <c r="C48">
-        <v>2884.8</v>
+        <v>0</v>
       </c>
       <c r="D48">
-        <v>0.05510043263941791</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -968,13 +968,13 @@
         <v>AAPL</v>
       </c>
       <c r="B49">
-        <v>238.03</v>
+        <v>213.32</v>
       </c>
       <c r="C49">
-        <v>3498.5</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>0.06682355733740863</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -982,13 +982,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B50">
-        <v>167.01</v>
+        <v>161.3</v>
       </c>
       <c r="C50">
-        <v>2020.3</v>
+        <v>0</v>
       </c>
       <c r="D50">
-        <v>0.03858886880058495</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -996,13 +996,13 @@
         <v>AMZN</v>
       </c>
       <c r="B51">
-        <v>205.02</v>
+        <v>190.2</v>
       </c>
       <c r="C51">
-        <v>2200.9</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>0.042037425561212205</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1010,13 +1010,13 @@
         <v>META</v>
       </c>
       <c r="B52">
-        <v>655.05</v>
+        <v>572.21</v>
       </c>
       <c r="C52">
-        <v>1651.4</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>0.0315419070226463</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1024,13 +1024,13 @@
         <v>TSLA</v>
       </c>
       <c r="B53">
-        <v>284.65</v>
+        <v>280.52</v>
       </c>
       <c r="C53">
-        <v>1068.1</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>0.02040167748110477</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1038,15 +1038,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C54">
-        <v>16101</v>
+        <v>0</v>
       </c>
       <c r="D54">
-        <v>0.3075359656728021</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>April 2025</v>
+        <v>June 2025</v>
       </c>
     </row>
     <row r="57">
@@ -1068,13 +1068,13 @@
         <v>NVDA</v>
       </c>
       <c r="B58">
-        <v>110.15</v>
+        <v>137.38</v>
       </c>
       <c r="C58">
-        <v>2681.8</v>
+        <v>0</v>
       </c>
       <c r="D58">
-        <v>0.05339503390497378</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -1082,13 +1082,13 @@
         <v>MSFT</v>
       </c>
       <c r="B59">
-        <v>382.19</v>
+        <v>461.97</v>
       </c>
       <c r="C59">
-        <v>2838</v>
+        <v>0</v>
       </c>
       <c r="D59">
-        <v>0.05650456435770747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1096,13 +1096,13 @@
         <v>AAPL</v>
       </c>
       <c r="B60">
-        <v>223.19</v>
+        <v>201.7</v>
       </c>
       <c r="C60">
-        <v>3280.4</v>
+        <v>0</v>
       </c>
       <c r="D60">
-        <v>0.06531330597781751</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -1110,13 +1110,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B61">
-        <v>157.07</v>
+        <v>169.03</v>
       </c>
       <c r="C61">
-        <v>1900.1</v>
+        <v>0</v>
       </c>
       <c r="D61">
-        <v>0.03783048273057432</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1124,13 +1124,13 @@
         <v>AMZN</v>
       </c>
       <c r="B62">
-        <v>192.17</v>
+        <v>206.65</v>
       </c>
       <c r="C62">
-        <v>2062.9</v>
+        <v>0</v>
       </c>
       <c r="D62">
-        <v>0.041072817181503976</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -1138,13 +1138,13 @@
         <v>META</v>
       </c>
       <c r="B63">
-        <v>586</v>
+        <v>670.9</v>
       </c>
       <c r="C63">
-        <v>1477.3</v>
+        <v>0</v>
       </c>
       <c r="D63">
-        <v>0.02941305624329163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1152,13 +1152,13 @@
         <v>TSLA</v>
       </c>
       <c r="B64">
-        <v>268.46</v>
+        <v>342.69</v>
       </c>
       <c r="C64">
-        <v>1007.4</v>
+        <v>0</v>
       </c>
       <c r="D64">
-        <v>0.020056876668653946</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -1166,15 +1166,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C65">
-        <v>15247.9</v>
+        <v>0</v>
       </c>
       <c r="D65">
-        <v>0.30358613706452264</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>May 2025</v>
+        <v>July 2025</v>
       </c>
     </row>
     <row r="68">
@@ -1196,13 +1196,13 @@
         <v>NVDA</v>
       </c>
       <c r="B69">
-        <v>111.61</v>
+        <v>153.3</v>
       </c>
       <c r="C69">
-        <v>2717.4</v>
+        <v>0</v>
       </c>
       <c r="D69">
-        <v>0.05451846630102624</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -1210,13 +1210,13 @@
         <v>MSFT</v>
       </c>
       <c r="B70">
-        <v>425.4</v>
+        <v>492.05</v>
       </c>
       <c r="C70">
-        <v>3158.9</v>
+        <v>0</v>
       </c>
       <c r="D70">
-        <v>0.06337614930315627</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1224,13 +1224,13 @@
         <v>AAPL</v>
       </c>
       <c r="B71">
-        <v>213.32</v>
+        <v>207.82</v>
       </c>
       <c r="C71">
-        <v>3135.4</v>
+        <v>0</v>
       </c>
       <c r="D71">
-        <v>0.06290463986676066</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -1238,13 +1238,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B72">
-        <v>161.3</v>
+        <v>175.84</v>
       </c>
       <c r="C72">
-        <v>1951.2</v>
+        <v>0</v>
       </c>
       <c r="D72">
-        <v>0.039147781434829075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -1252,13 +1252,13 @@
         <v>AMZN</v>
       </c>
       <c r="B73">
-        <v>190.2</v>
+        <v>220.46</v>
       </c>
       <c r="C73">
-        <v>2041.8</v>
+        <v>0</v>
       </c>
       <c r="D73">
-        <v>0.040964114557301146</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1266,13 +1266,13 @@
         <v>META</v>
       </c>
       <c r="B74">
-        <v>572.21</v>
+        <v>719.22</v>
       </c>
       <c r="C74">
-        <v>1442.5</v>
+        <v>0</v>
       </c>
       <c r="D74">
-        <v>0.028941574726441665</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -1280,13 +1280,13 @@
         <v>TSLA</v>
       </c>
       <c r="B75">
-        <v>280.52</v>
+        <v>300.71</v>
       </c>
       <c r="C75">
-        <v>1052.6</v>
+        <v>0</v>
       </c>
       <c r="D75">
-        <v>0.021118920018962154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1294,15 +1294,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C76">
-        <v>15499.8</v>
+        <v>0</v>
       </c>
       <c r="D76">
-        <v>0.3109716462084772</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>June 2025</v>
+        <v>August 2025</v>
       </c>
     </row>
     <row r="79">
@@ -1324,13 +1324,13 @@
         <v>NVDA</v>
       </c>
       <c r="B80">
-        <v>137.38</v>
+        <v>173.72</v>
       </c>
       <c r="C80">
-        <v>3344.8</v>
+        <v>0</v>
       </c>
       <c r="D80">
-        <v>0.06295880121805197</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
@@ -1338,13 +1338,13 @@
         <v>MSFT</v>
       </c>
       <c r="B81">
-        <v>461.97</v>
+        <v>524.11</v>
       </c>
       <c r="C81">
-        <v>3430.4</v>
+        <v>0</v>
       </c>
       <c r="D81">
-        <v>0.06457055911880254</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -1352,13 +1352,13 @@
         <v>AAPL</v>
       </c>
       <c r="B82">
-        <v>201.7</v>
+        <v>202.38</v>
       </c>
       <c r="C82">
-        <v>2964.6</v>
+        <v>0</v>
       </c>
       <c r="D82">
-        <v>0.05580195124854954</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -1366,13 +1366,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B83">
-        <v>169.03</v>
+        <v>189.13</v>
       </c>
       <c r="C83">
-        <v>2044.8</v>
+        <v>0</v>
       </c>
       <c r="D83">
-        <v>0.03848832144017101</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -1380,13 +1380,13 @@
         <v>AMZN</v>
       </c>
       <c r="B84">
-        <v>206.65</v>
+        <v>214.75</v>
       </c>
       <c r="C84">
-        <v>2218.4</v>
+        <v>0</v>
       </c>
       <c r="D84">
-        <v>0.04175619013332163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -1394,13 +1394,13 @@
         <v>META</v>
       </c>
       <c r="B85">
-        <v>670.9</v>
+        <v>750.01</v>
       </c>
       <c r="C85">
-        <v>1691.3</v>
+        <v>0</v>
       </c>
       <c r="D85">
-        <v>0.03183588363426788</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -1408,13 +1408,13 @@
         <v>TSLA</v>
       </c>
       <c r="B86">
-        <v>342.69</v>
+        <v>302.63</v>
       </c>
       <c r="C86">
-        <v>1285.9</v>
+        <v>0</v>
       </c>
       <c r="D86">
-        <v>0.02420481291007333</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
@@ -1422,15 +1422,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C87">
-        <v>16980.2</v>
+        <v>0</v>
       </c>
       <c r="D87">
-        <v>0.3196165197032379</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>July 2025</v>
+        <v>September 2025</v>
       </c>
     </row>
     <row r="90">
@@ -1452,13 +1452,13 @@
         <v>NVDA</v>
       </c>
       <c r="B91">
-        <v>153.3</v>
+        <v>170.78</v>
       </c>
       <c r="C91">
-        <v>3732.4</v>
+        <v>0</v>
       </c>
       <c r="D91">
-        <v>0.06720882215989255</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -1466,13 +1466,13 @@
         <v>MSFT</v>
       </c>
       <c r="B92">
-        <v>492.05</v>
+        <v>505.12</v>
       </c>
       <c r="C92">
-        <v>3653.8</v>
+        <v>0</v>
       </c>
       <c r="D92">
-        <v>0.06579322817362217</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -1480,13 +1480,13 @@
         <v>AAPL</v>
       </c>
       <c r="B93">
-        <v>207.82</v>
+        <v>229.72</v>
       </c>
       <c r="C93">
-        <v>3054.5</v>
+        <v>0</v>
       </c>
       <c r="D93">
-        <v>0.055002451626620034</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -1494,13 +1494,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B94">
-        <v>175.84</v>
+        <v>211.35</v>
       </c>
       <c r="C94">
-        <v>2127.1</v>
+        <v>0</v>
       </c>
       <c r="D94">
-        <v>0.03830311081425009</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -1508,13 +1508,13 @@
         <v>AMZN</v>
       </c>
       <c r="B95">
-        <v>220.46</v>
+        <v>225.34</v>
       </c>
       <c r="C95">
-        <v>2366.6</v>
+        <v>0</v>
       </c>
       <c r="D95">
-        <v>0.04261539165957815</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -1522,13 +1522,13 @@
         <v>META</v>
       </c>
       <c r="B96">
-        <v>719.22</v>
+        <v>735.11</v>
       </c>
       <c r="C96">
-        <v>1813.1</v>
+        <v>0</v>
       </c>
       <c r="D96">
-        <v>0.032649161880347714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -1536,13 +1536,13 @@
         <v>TSLA</v>
       </c>
       <c r="B97">
-        <v>300.71</v>
+        <v>329.36</v>
       </c>
       <c r="C97">
-        <v>1128.4</v>
+        <v>0</v>
       </c>
       <c r="D97">
-        <v>0.020318860659609094</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -1550,15 +1550,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C98">
-        <v>17876</v>
+        <v>0</v>
       </c>
       <c r="D98">
-        <v>0.3218910269739198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>August 2025</v>
+        <v>October 2025</v>
       </c>
     </row>
     <row r="101">
@@ -1580,13 +1580,13 @@
         <v>NVDA</v>
       </c>
       <c r="B102">
-        <v>173.72</v>
+        <v>187.24</v>
       </c>
       <c r="C102">
-        <v>4229.6</v>
+        <v>0</v>
       </c>
       <c r="D102">
-        <v>0.07454607206092621</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -1594,13 +1594,13 @@
         <v>MSFT</v>
       </c>
       <c r="B103">
-        <v>524.11</v>
+        <v>519.71</v>
       </c>
       <c r="C103">
-        <v>3891.8</v>
+        <v>0</v>
       </c>
       <c r="D103">
-        <v>0.06859385712344067</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -1608,13 +1608,13 @@
         <v>AAPL</v>
       </c>
       <c r="B104">
-        <v>202.38</v>
+        <v>255.45</v>
       </c>
       <c r="C104">
-        <v>2974.6</v>
+        <v>0</v>
       </c>
       <c r="D104">
-        <v>0.052426771494219315</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -1622,13 +1622,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B105">
-        <v>189.13</v>
+        <v>244.9</v>
       </c>
       <c r="C105">
-        <v>2287.9</v>
+        <v>0</v>
       </c>
       <c r="D105">
-        <v>0.040324374067196835</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
@@ -1636,13 +1636,13 @@
         <v>AMZN</v>
       </c>
       <c r="B106">
-        <v>214.75</v>
+        <v>220.63</v>
       </c>
       <c r="C106">
-        <v>2305.3</v>
+        <v>0</v>
       </c>
       <c r="D106">
-        <v>0.040631294641370906</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -1650,13 +1650,13 @@
         <v>META</v>
       </c>
       <c r="B107">
-        <v>750.01</v>
+        <v>717.34</v>
       </c>
       <c r="C107">
-        <v>1890.8</v>
+        <v>0</v>
       </c>
       <c r="D107">
-        <v>0.033324848131571445</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -1664,13 +1664,13 @@
         <v>TSLA</v>
       </c>
       <c r="B108">
-        <v>302.63</v>
+        <v>459.46</v>
       </c>
       <c r="C108">
-        <v>1135.6</v>
+        <v>0</v>
       </c>
       <c r="D108">
-        <v>0.020014940287187883</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -1678,15 +1678,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C109">
-        <v>18715.6</v>
+        <v>0</v>
       </c>
       <c r="D109">
-        <v>0.3298621578059132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>September 2025</v>
+        <v>November 2025</v>
       </c>
     </row>
     <row r="112">
@@ -1708,13 +1708,13 @@
         <v>NVDA</v>
       </c>
       <c r="B113">
-        <v>170.78</v>
+        <v>206.88</v>
       </c>
       <c r="C113">
-        <v>4158</v>
+        <v>0</v>
       </c>
       <c r="D113">
-        <v>0.07241461186451607</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
@@ -1722,13 +1722,13 @@
         <v>MSFT</v>
       </c>
       <c r="B114">
-        <v>505.12</v>
+        <v>517.03</v>
       </c>
       <c r="C114">
-        <v>3750.8</v>
+        <v>0</v>
       </c>
       <c r="D114">
-        <v>0.06532382564354466</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115">
@@ -1736,13 +1736,13 @@
         <v>AAPL</v>
       </c>
       <c r="B115">
-        <v>229.72</v>
+        <v>269.05</v>
       </c>
       <c r="C115">
-        <v>3376.4</v>
+        <v>0</v>
       </c>
       <c r="D115">
-        <v>0.058802877963955745</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116">
@@ -1750,13 +1750,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B116">
-        <v>211.35</v>
+        <v>283.72</v>
       </c>
       <c r="C116">
-        <v>2556.7</v>
+        <v>0</v>
       </c>
       <c r="D116">
-        <v>0.04452702975580989</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -1764,13 +1764,13 @@
         <v>AMZN</v>
       </c>
       <c r="B117">
-        <v>225.34</v>
+        <v>254</v>
       </c>
       <c r="C117">
-        <v>2419</v>
+        <v>0</v>
       </c>
       <c r="D117">
-        <v>0.042128891399379656</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -1778,13 +1778,13 @@
         <v>META</v>
       </c>
       <c r="B118">
-        <v>735.11</v>
+        <v>637.71</v>
       </c>
       <c r="C118">
-        <v>1853.2</v>
+        <v>0</v>
       </c>
       <c r="D118">
-        <v>0.03227510779350659</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -1792,13 +1792,13 @@
         <v>TSLA</v>
       </c>
       <c r="B119">
-        <v>329.36</v>
+        <v>468.37</v>
       </c>
       <c r="C119">
-        <v>1235.9</v>
+        <v>0</v>
       </c>
       <c r="D119">
-        <v>0.021524219321961406</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -1806,15 +1806,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C120">
-        <v>19350</v>
+        <v>0</v>
       </c>
       <c r="D120">
-        <v>0.336996563742674</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>October 2025</v>
+        <v>December 2025</v>
       </c>
     </row>
     <row r="123">
@@ -1836,13 +1836,13 @@
         <v>NVDA</v>
       </c>
       <c r="B124">
-        <v>187.24</v>
+        <v>179.92</v>
       </c>
       <c r="C124">
-        <v>4558.7</v>
+        <v>0</v>
       </c>
       <c r="D124">
-        <v>0.07615438836911599</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -1850,13 +1850,13 @@
         <v>MSFT</v>
       </c>
       <c r="B125">
-        <v>519.71</v>
+        <v>486.74</v>
       </c>
       <c r="C125">
-        <v>3859.2</v>
+        <v>0</v>
       </c>
       <c r="D125">
-        <v>0.0644681533775499</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -1864,13 +1864,13 @@
         <v>AAPL</v>
       </c>
       <c r="B126">
-        <v>255.45</v>
+        <v>283.1</v>
       </c>
       <c r="C126">
-        <v>3754.6</v>
+        <v>0</v>
       </c>
       <c r="D126">
-        <v>0.06272096940724874</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">
@@ -1878,13 +1878,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B127">
-        <v>244.9</v>
+        <v>314.89</v>
       </c>
       <c r="C127">
-        <v>2962.6</v>
+        <v>0</v>
       </c>
       <c r="D127">
-        <v>0.049489985154853276</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
@@ -1892,13 +1892,13 @@
         <v>AMZN</v>
       </c>
       <c r="B128">
-        <v>220.63</v>
+        <v>233.88</v>
       </c>
       <c r="C128">
-        <v>2368.4</v>
+        <v>0</v>
       </c>
       <c r="D128">
-        <v>0.039565204139548324</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -1906,13 +1906,13 @@
         <v>META</v>
       </c>
       <c r="B129">
-        <v>717.34</v>
+        <v>640.87</v>
       </c>
       <c r="C129">
-        <v>1808.4</v>
+        <v>0</v>
       </c>
       <c r="D129">
-        <v>0.03020977788937343</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -1920,13 +1920,13 @@
         <v>TSLA</v>
       </c>
       <c r="B130">
-        <v>459.46</v>
+        <v>430.14</v>
       </c>
       <c r="C130">
-        <v>1724.1</v>
+        <v>0</v>
       </c>
       <c r="D130">
-        <v>0.028801251680996544</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -1934,15 +1934,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C131">
-        <v>21036</v>
+        <v>0</v>
       </c>
       <c r="D131">
-        <v>0.35140973001868625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>November 2025</v>
+        <v>January 2026</v>
       </c>
     </row>
     <row r="134">
@@ -1964,13 +1964,13 @@
         <v>NVDA</v>
       </c>
       <c r="B135">
-        <v>206.88</v>
+        <v>188.85</v>
       </c>
       <c r="C135">
-        <v>5036.9</v>
+        <v>0</v>
       </c>
       <c r="D135">
-        <v>0.08213447248644803</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -1978,13 +1978,13 @@
         <v>MSFT</v>
       </c>
       <c r="B136">
-        <v>517.03</v>
+        <v>472.94</v>
       </c>
       <c r="C136">
-        <v>3839.3</v>
+        <v>0</v>
       </c>
       <c r="D136">
-        <v>0.0626052237012684</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -1992,13 +1992,13 @@
         <v>AAPL</v>
       </c>
       <c r="B137">
-        <v>269.05</v>
+        <v>271.01</v>
       </c>
       <c r="C137">
-        <v>3954.5</v>
+        <v>0</v>
       </c>
       <c r="D137">
-        <v>0.0644837821548035</v>
+        <v>0</v>
       </c>
     </row>
     <row r="138">
@@ -2006,13 +2006,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B138">
-        <v>283.72</v>
+        <v>315.15</v>
       </c>
       <c r="C138">
-        <v>3432.2</v>
+        <v>0</v>
       </c>
       <c r="D138">
-        <v>0.05596663135977788</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -2020,13 +2020,13 @@
         <v>AMZN</v>
       </c>
       <c r="B139">
-        <v>254</v>
+        <v>226.5</v>
       </c>
       <c r="C139">
-        <v>2726.7</v>
+        <v>0</v>
       </c>
       <c r="D139">
-        <v>0.04446243241248235</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -2034,13 +2034,13 @@
         <v>META</v>
       </c>
       <c r="B140">
-        <v>637.71</v>
+        <v>650.41</v>
       </c>
       <c r="C140">
-        <v>1607.7</v>
+        <v>0</v>
       </c>
       <c r="D140">
-        <v>0.026215393133655042</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
@@ -2048,13 +2048,13 @@
         <v>TSLA</v>
       </c>
       <c r="B141">
-        <v>468.37</v>
+        <v>438.07</v>
       </c>
       <c r="C141">
-        <v>1757.5</v>
+        <v>0</v>
       </c>
       <c r="D141">
-        <v>0.028659155747857726</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -2062,15 +2062,15 @@
         <v>TOTAL</v>
       </c>
       <c r="C142">
-        <v>22354.7</v>
+        <v>0</v>
       </c>
       <c r="D142">
-        <v>0.36452709099629294</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>December 2025</v>
+        <v>February 2026</v>
       </c>
     </row>
     <row r="145">
@@ -2092,13 +2092,13 @@
         <v>NVDA</v>
       </c>
       <c r="B146" s="1">
-        <v>179.92</v>
+        <v>185.61</v>
       </c>
       <c r="C146" s="2">
-        <v>4380.5</v>
+        <v>0</v>
       </c>
       <c r="D146" s="3">
-        <v>0.07184343084835443</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
@@ -2106,13 +2106,13 @@
         <v>MSFT</v>
       </c>
       <c r="B147" s="1">
-        <v>486.74</v>
+        <v>423.37</v>
       </c>
       <c r="C147" s="2">
-        <v>3614.4</v>
+        <v>0</v>
       </c>
       <c r="D147" s="3">
-        <v>0.05927785829233961</v>
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -2120,13 +2120,13 @@
         <v>AAPL</v>
       </c>
       <c r="B148" s="1">
-        <v>283.1</v>
+        <v>270.01</v>
       </c>
       <c r="C148" s="2">
-        <v>4161</v>
+        <v>0</v>
       </c>
       <c r="D148" s="3">
-        <v>0.06824299450538433</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149">
@@ -2134,13 +2134,13 @@
         <v>GOOGL</v>
       </c>
       <c r="B149" s="1">
-        <v>314.89</v>
+        <v>343.69</v>
       </c>
       <c r="C149" s="2">
-        <v>3809.2</v>
+        <v>0</v>
       </c>
       <c r="D149" s="3">
-        <v>0.06247392253795553</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -2148,13 +2148,13 @@
         <v>AMZN</v>
       </c>
       <c r="B150" s="1">
-        <v>233.88</v>
+        <v>242.96</v>
       </c>
       <c r="C150" s="2">
-        <v>2510.7</v>
+        <v>0</v>
       </c>
       <c r="D150" s="3">
-        <v>0.04117686389540775</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
@@ -2162,13 +2162,13 @@
         <v>META</v>
       </c>
       <c r="B151" s="1">
-        <v>640.87</v>
+        <v>706.41</v>
       </c>
       <c r="C151" s="2">
-        <v>1615.6</v>
+        <v>0</v>
       </c>
       <c r="D151" s="3">
-        <v>0.026497429343704814</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -2176,13 +2176,13 @@
         <v>TSLA</v>
       </c>
       <c r="B152" s="1">
-        <v>430.14</v>
+        <v>421.81</v>
       </c>
       <c r="C152" s="2">
-        <v>1614.1</v>
+        <v>0</v>
       </c>
       <c r="D152" s="3">
-        <v>0.026471883574073173</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -2190,10 +2190,10 @@
         <v>TOTAL</v>
       </c>
       <c r="C153" s="2">
-        <v>21705.4</v>
+        <v>0</v>
       </c>
       <c r="D153" s="3">
-        <v>0.35598438299721963</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update stock exports (VPS cron)
</commit_message>
<xml_diff>
--- a/projects/all-in/exports/MagSeven.xlsx
+++ b/projects/all-in/exports/MagSeven.xlsx
@@ -66,8 +66,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="61" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -399,13 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
-  <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -663,13 +660,142 @@
         <v>0.34851314349008283</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>March 2026</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Ticker</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Share Price</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Mkt Cap ($B)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>% of S&amp;P 500</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>NVDA</v>
+      </c>
+      <c r="B26" s="1">
+        <v>177.19</v>
+      </c>
+      <c r="C26" s="2">
+        <v>4306.6</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0.06995102427438445</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>MSFT</v>
+      </c>
+      <c r="B27" s="1">
+        <v>392.74</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2916.3</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.047369376978609094</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>AAPL</v>
+      </c>
+      <c r="B28" s="1">
+        <v>264.18</v>
+      </c>
+      <c r="C28" s="2">
+        <v>3882.9</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0.06306889213311066</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>GOOGL</v>
+      </c>
+      <c r="B29" s="1">
+        <v>311.76</v>
+      </c>
+      <c r="C29" s="2">
+        <v>3771.4</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0.06125722542380096</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>AMZN</v>
+      </c>
+      <c r="B30" s="1">
+        <v>210</v>
+      </c>
+      <c r="C30" s="2">
+        <v>2254.3</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0.036616545845062215</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>META</v>
+      </c>
+      <c r="B31" s="1">
+        <v>648.18</v>
+      </c>
+      <c r="C31" s="2">
+        <v>1634.1</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0.026541562869829595</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>TSLA</v>
+      </c>
+      <c r="B32" s="1">
+        <v>402.51</v>
+      </c>
+      <c r="C32" s="2">
+        <v>1510.4</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0.02453289131451177</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>TOTAL</v>
+      </c>
+      <c r="C33" s="2">
+        <v>20276</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0.32933751883930884</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A24:D24"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>